<commit_message>
correction on input electricity mix
</commit_message>
<xml_diff>
--- a/inventories/lci-FE2050.xlsx
+++ b/inventories/lci-FE2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\RTE_scenarios\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C398A2FA-30DE-4764-A9BE-ECCD79E121F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB70237-5422-41BC-B016-5F2379F27E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="140">
   <si>
     <t>Database</t>
   </si>
@@ -452,10 +452,13 @@
     <t>kilometer</t>
   </si>
   <si>
-    <t>input mix for storage, FE2050</t>
+    <t>intermediate activity to ease the change of input mix for storage and release technologies</t>
   </si>
   <si>
-    <t>intermediate activity to ease the change of input mix for storage and release technologies</t>
+    <t>input electricity mix for storage, FE2050</t>
+  </si>
+  <si>
+    <t>input eletricity mix for storage, FE2050</t>
   </si>
 </sst>
 </file>
@@ -25858,7 +25861,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="9"/>
@@ -25890,7 +25893,7 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
@@ -25993,7 +25996,7 @@
     </row>
     <row r="28" spans="1:1019 1025:2043 2049:3067 3073:4091 4097:5115 5121:6139 6145:7163 7169:8187 8193:9211 9217:10235 10241:11259 11265:12283 12289:13307 13313:14331 14337:15355 15361:16379">
       <c r="A28" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B28" s="19">
         <v>1</v>
@@ -32350,7 +32353,7 @@
     </row>
     <row r="40" spans="1:11">
       <c r="A40" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B40" s="19">
         <f>1*1.12*1.15</f>
@@ -32601,7 +32604,7 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B54" s="19">
         <v>1.25125</v>
@@ -33686,7 +33689,7 @@
     </row>
     <row r="108" spans="1:20" s="25" customFormat="1" ht="15.5">
       <c r="A108" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B108" s="44">
         <v>54</v>
@@ -33999,7 +34002,7 @@
     </row>
     <row r="125" spans="1:14">
       <c r="A125" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B125">
         <v>1.33</v>

</xml_diff>

<commit_message>
? minor change in inventories file ?
</commit_message>
<xml_diff>
--- a/inventories/lci-FE2050.xlsx
+++ b/inventories/lci-FE2050.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jschlesinger\0.Joanna\RTE_scenarios\inventories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB70237-5422-41BC-B016-5F2379F27E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A867B74F-764C-49FC-8076-D1E74DFF5FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="139">
   <si>
     <t>Database</t>
   </si>
@@ -456,9 +456,6 @@
   </si>
   <si>
     <t>input electricity mix for storage, FE2050</t>
-  </si>
-  <si>
-    <t>input eletricity mix for storage, FE2050</t>
   </si>
 </sst>
 </file>
@@ -32604,7 +32601,7 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B54" s="19">
         <v>1.25125</v>

</xml_diff>